<commit_message>
Stable v1: finalize sales and stock matching pipeline
</commit_message>
<xml_diff>
--- a/data/06.04.26 инвентаризация(полн).xlsx
+++ b/data/06.04.26 инвентаризация(полн).xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ЭтаКнига" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\SVO\Склад\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\SVO\AI\SVO_MATCH_ENGINE\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{490A2929-99D4-4409-9590-9AE572FFCBC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A496BA7D-B6ED-4E6B-AE02-3583678B43F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{BD2D0025-E6D5-42F3-8FFB-3B68B9570BCD}"/>
   </bookViews>

</xml_diff>